<commit_message>
Completed Market Pulse v1.0
</commit_message>
<xml_diff>
--- a/Output/Dashboard.xlsx
+++ b/Output/Dashboard.xlsx
@@ -11,7 +11,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Option Buying" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Long Term" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Market Pulse'!$A$4:$H$7</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -19,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,16 +33,49 @@
       <b val="1"/>
       <sz val="16"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="18"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C6EFCE"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -48,13 +83,29 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -420,80 +471,211 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:H12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>AQSD MARKET PULSE</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>AQSD PROFESSIONAL - MARKET PULSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Last Updated</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>14-07-2026 12:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Index</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t>Close</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>EMA20</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>EMA50</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>RSI</t>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>RSI14</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Daily %</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>Weekly %</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>Trend</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>NIFTY</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>24090</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>24035.06</v>
+      </c>
+      <c r="D5" s="5" t="n">
+        <v>23949.68</v>
+      </c>
+      <c r="E5" s="5" t="n">
+        <v>52.62</v>
+      </c>
+      <c r="F5" s="5" t="n">
+        <v>-0.5</v>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>-1.27</v>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>BANKNIFTY</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>57486.45</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>57393.91</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>56597.64</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>53.04</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>-1.11</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>-1.23</v>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>INDIA VIX</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>13.65</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>13.46</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>14.93</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>48.99</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>17.12</v>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>Neutral</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>Market Bias</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>🟢 BULLISH</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>BULLISH</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>Confidence</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>Strategy</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="B12" t="inlineStr">
         <is>
           <t>CALL BUYING</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A4:H7"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>